<commit_message>
Justify choice of 10 and some EDA
</commit_message>
<xml_diff>
--- a/Data/BUS/Cost_index_18.xlsx
+++ b/Data/BUS/Cost_index_18.xlsx
@@ -450,7 +450,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1.841896475196469</v>
+        <v>1.84930949412904</v>
       </c>
     </row>
     <row r="3">
@@ -463,7 +463,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>3.075892816194178</v>
+        <v>3.075867121037544</v>
       </c>
     </row>
     <row r="4">
@@ -476,7 +476,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>4.273722181321732</v>
+        <v>4.27639364943454</v>
       </c>
     </row>
     <row r="5">
@@ -489,7 +489,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>5.492940843558475</v>
+        <v>5.49274023187377</v>
       </c>
     </row>
     <row r="6">
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1.972499863130221</v>
+        <v>1.978903614925749</v>
       </c>
     </row>
     <row r="7">
@@ -515,7 +515,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>5.070724318289583</v>
+        <v>5.082911944550688</v>
       </c>
     </row>
     <row r="8">
@@ -528,7 +528,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>3.781400042572422</v>
+        <v>3.818203773844363</v>
       </c>
     </row>
     <row r="9">
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2.125092046304117</v>
+        <v>2.114631448180023</v>
       </c>
     </row>
     <row r="10">
@@ -554,7 +554,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2.588575967445989</v>
+        <v>2.585819340022317</v>
       </c>
     </row>
     <row r="11">
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2.164483808755148</v>
+        <v>2.169578909493137</v>
       </c>
     </row>
     <row r="12">
@@ -580,7 +580,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2.953228486709973</v>
+        <v>2.955856734516588</v>
       </c>
     </row>
     <row r="13">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1.782158958899993</v>
+        <v>1.776562611907709</v>
       </c>
     </row>
     <row r="14">
@@ -606,7 +606,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3.696629360263973</v>
+        <v>3.694651283975074</v>
       </c>
     </row>
     <row r="15">
@@ -619,7 +619,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2.247986187755254</v>
+        <v>2.218062621383034</v>
       </c>
     </row>
     <row r="16">
@@ -632,7 +632,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>5.55856961178666</v>
+        <v>5.574087662420545</v>
       </c>
     </row>
     <row r="17">
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>2.010924353242042</v>
+        <v>2.010126630445508</v>
       </c>
     </row>
     <row r="18">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2.126160760024053</v>
+        <v>2.117823541057404</v>
       </c>
     </row>
     <row r="19">
@@ -671,7 +671,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>3.190044235911958</v>
+        <v>3.17919440991437</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Justify choice of 10 and some EDA finish EDA
</commit_message>
<xml_diff>
--- a/Data/BUS/Cost_index_18.xlsx
+++ b/Data/BUS/Cost_index_18.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>